<commit_message>
chore: run 2026-09-13 21:49 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_13_09_2026.xlsx
+++ b/logs/Consolidado_13_09_2026.xlsx
@@ -657,10 +657,10 @@
         <v>154</v>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>9</v>
@@ -676,10 +676,10 @@
         <v>69</v>
       </c>
       <c r="C3" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
@@ -695,10 +695,10 @@
         <v>79</v>
       </c>
       <c r="C4" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>9</v>
@@ -714,10 +714,10 @@
         <v>68</v>
       </c>
       <c r="C5" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
@@ -733,10 +733,10 @@
         <v>48</v>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>5</v>
@@ -752,10 +752,10 @@
         <v>102</v>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>6</v>
@@ -5402,38 +5402,38 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="7" t="inlineStr">
+      <c r="A124" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="B124" s="7" t="inlineStr">
+      <c r="B124" s="3" t="inlineStr">
         <is>
           <t>Cleanance Micellar Water
 Água Micelar Limpeza Pele Oleosa e Acneica</t>
         </is>
       </c>
-      <c r="C124" s="7" t="inlineStr">
+      <c r="C124" s="3" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="D124" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E124" s="7" t="inlineStr">
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
         <is>
           <t>6552597</t>
         </is>
       </c>
-      <c r="F124" s="7" t="inlineStr">
+      <c r="F124" s="3" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
       </c>
-      <c r="G124" s="7" t="inlineStr">
+      <c r="G124" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cleanance-micellar-water-443919.html</t>
         </is>
@@ -8404,38 +8404,38 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="7" t="inlineStr">
+      <c r="A205" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="B205" s="7" t="inlineStr">
+      <c r="B205" s="5" t="inlineStr">
         <is>
           <t>Sun Care Lotion 100% Invisible SPF50
 Protetor Solar Leite Corpo Pele Sensível</t>
         </is>
       </c>
-      <c r="C205" s="7" t="inlineStr">
+      <c r="C205" s="5" t="inlineStr">
         <is>
           <t>250 ml</t>
         </is>
       </c>
-      <c r="D205" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E205" s="7" t="inlineStr">
+      <c r="D205" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E205" s="5" t="inlineStr">
         <is>
           <t>8384283</t>
         </is>
       </c>
-      <c r="F205" s="7" t="inlineStr">
+      <c r="F205" s="5" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
       </c>
-      <c r="G205" s="7" t="inlineStr">
+      <c r="G205" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/sun-care-lotion-100-invisible-spf50-396990.html</t>
         </is>
@@ -14242,38 +14242,38 @@
       </c>
     </row>
     <row r="362">
-      <c r="A362" s="7" t="inlineStr">
+      <c r="A362" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B362" s="7" t="inlineStr">
+      <c r="B362" s="3" t="inlineStr">
         <is>
           <t>Flax Volume Fine Hair Shampoo
 Champô Fibras de Linho BIO Volume Cabelo Fino</t>
         </is>
       </c>
-      <c r="C362" s="7" t="inlineStr">
+      <c r="C362" s="3" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="D362" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E362" s="7" t="inlineStr">
+      <c r="D362" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E362" s="3" t="inlineStr">
         <is>
           <t>5418515</t>
         </is>
       </c>
-      <c r="F362" s="7" t="inlineStr">
+      <c r="F362" s="3" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
       </c>
-      <c r="G362" s="7" t="inlineStr">
+      <c r="G362" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/flax-volume-fine-hair-shampoo-343984.html</t>
         </is>
@@ -15371,38 +15371,38 @@
       </c>
     </row>
     <row r="392">
-      <c r="A392" s="7" t="inlineStr">
+      <c r="A392" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B392" s="7" t="inlineStr">
+      <c r="B392" s="3" t="inlineStr">
         <is>
           <t>Prickly Pear 72h Hydration &amp; Shine Shampoo
 Champô Figo da Índia Hidratante Cabelo Baço</t>
         </is>
       </c>
-      <c r="C392" s="7" t="inlineStr">
+      <c r="C392" s="3" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="D392" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E392" s="7" t="inlineStr">
+      <c r="D392" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E392" s="3" t="inlineStr">
         <is>
           <t>8067425</t>
         </is>
       </c>
-      <c r="F392" s="7" t="inlineStr">
+      <c r="F392" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G392" s="7" t="inlineStr">
+      <c r="G392" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/prickly-pear-72h-hydration-and-shine-shampoo-355576.html</t>
         </is>
@@ -19345,40 +19345,40 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Anti-Imperfection Fluid SPF50
 Protetor Solar Fluido Rosto Anti-Imperfeições
 40 ml</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/anti-imperfection-fluid-spf50-8337858.html</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>8337858</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
@@ -20315,40 +20315,40 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Cleanance Comedomed Peeling
 Creme Peeling Redutor Borbulhas Pele Acneica
 40 ml</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cleanance-comedomed-peeling-8152746.html</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr"/>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>8152746</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
@@ -20638,43 +20638,43 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>Cleanance Micellar Water
 Água Micelar Limpeza Pele Oleosa e Acneica</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cleanance-micellar-water-443919.html</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>6552597</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
@@ -23566,43 +23566,43 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B110" s="7" t="inlineStr">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C110" s="7" t="inlineStr">
+      <c r="C110" s="3" t="inlineStr">
         <is>
           <t>Sun Care Lotion 100% Invisible SPF50
 Protetor Solar Leite Corpo Pele Sensível</t>
         </is>
       </c>
-      <c r="D110" s="7" t="inlineStr">
+      <c r="D110" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/sun-care-lotion-100-invisible-spf50-396990.html</t>
         </is>
       </c>
-      <c r="E110" s="7" t="inlineStr">
+      <c r="E110" s="3" t="inlineStr">
         <is>
           <t>250 ml</t>
         </is>
       </c>
-      <c r="F110" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G110" s="7" t="inlineStr">
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
         <is>
           <t>8384283</t>
         </is>
       </c>
-      <c r="H110" s="7" t="inlineStr">
+      <c r="H110" s="3" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
@@ -24169,40 +24169,40 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B125" s="7" t="inlineStr">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C125" s="7" t="inlineStr">
+      <c r="C125" s="5" t="inlineStr">
         <is>
           <t>Sun Care Sunsimed KA UVB UVA Blue Light
 Protetor Solar Prevenção Queratose Actínica
 80 ml</t>
         </is>
       </c>
-      <c r="D125" s="7" t="inlineStr">
+      <c r="D125" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/sun-care-sunsimed-ka-uvb-uva-blue-light-8016030.html</t>
         </is>
       </c>
-      <c r="E125" s="7" t="inlineStr"/>
-      <c r="F125" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G125" s="7" t="inlineStr">
+      <c r="E125" s="5" t="inlineStr"/>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
         <is>
           <t>8016030</t>
         </is>
       </c>
-      <c r="H125" s="7" t="inlineStr">
+      <c r="H125" s="5" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
@@ -26304,40 +26304,40 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Bálsamo Emoliente Antiprurido Dexyane
 Bálsamo Antiprurido Pele Seca e Eczema Atópico
 400 ml</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/balsamo-emoliente-antiprurido-dexyane-5976214.html</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>5976214</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -27770,40 +27770,40 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>Keracnyl Mat 12H Oily Skin
 Gel Matificante Pele Oleosa Ação Anti-brilho
 30 ml</t>
         </is>
       </c>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/keracnyl-mat-12h-oily-skin-6037944.html</t>
         </is>
       </c>
-      <c r="E48" s="7" t="inlineStr"/>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
         <is>
           <t>6037944</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H48" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -27850,40 +27850,40 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>Keracnyl Repair Baume Lèvres
 Bálsamo Lábios Gretados e Danificados Acne
 15 ml</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/keracnyl-repair-baume-levres-5410512.html</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr"/>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr"/>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
         <is>
           <t>5410512</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H50" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -28130,40 +28130,40 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Kit Anaphase Anti-Hair Loss and Growth
 Champô Queda de Cabelo Reativa com Oferta
 1 un</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/kit-anaphase-anti-hair-loss-and-growth-8640386.html</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr"/>
-      <c r="F57" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>8640386</t>
         </is>
       </c>
-      <c r="H57" s="7" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
@@ -28610,40 +28610,40 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B69" s="7" t="inlineStr">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C69" s="7" t="inlineStr">
+      <c r="C69" s="3" t="inlineStr">
         <is>
           <t>Sabal Shampooing Traitant Sébo-Régulateur
 Champô Seborregulador Cabelo Oleoso
 200 ml</t>
         </is>
       </c>
-      <c r="D69" s="7" t="inlineStr">
+      <c r="D69" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/sabal-shampooing-traitant-sebo-regulateur-8471859.html</t>
         </is>
       </c>
-      <c r="E69" s="7" t="inlineStr"/>
-      <c r="F69" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G69" s="7" t="inlineStr">
+      <c r="E69" s="3" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
         <is>
           <t>8471859</t>
         </is>
       </c>
-      <c r="H69" s="7" t="inlineStr">
+      <c r="H69" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -28690,40 +28690,40 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C71" s="7" t="inlineStr">
+      <c r="C71" s="3" t="inlineStr">
         <is>
           <t>Sensinol Shampooing Physioprotecteur
 Champô Calmante Couro Cabeludo Sensível
 400 ml</t>
         </is>
       </c>
-      <c r="D71" s="7" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/sensinol-shampooing-physioprotecteur-7646502.html</t>
         </is>
       </c>
-      <c r="E71" s="7" t="inlineStr"/>
-      <c r="F71" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G71" s="7" t="inlineStr">
+      <c r="E71" s="3" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
         <is>
           <t>7646502</t>
         </is>
       </c>
-      <c r="H71" s="7" t="inlineStr">
+      <c r="H71" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -30252,43 +30252,43 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Flax Volume Fine Hair Shampoo
 Champô Fibras de Linho BIO Volume Cabelo Fino</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/flax-volume-fine-hair-shampoo-343984.html</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>5418515</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
@@ -31820,39 +31820,39 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C71" s="7" t="inlineStr">
+      <c r="C71" s="3" t="inlineStr">
         <is>
           <t>Pack Champô Antiqueda Quinina Edelvaisse Bio
 400 ml + 400 ml</t>
         </is>
       </c>
-      <c r="D71" s="7" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/pack-champo-antiqueda-quinina-edelvaisse-bio-7834046.html</t>
         </is>
       </c>
-      <c r="E71" s="7" t="inlineStr"/>
-      <c r="F71" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G71" s="7" t="inlineStr">
+      <c r="E71" s="3" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
         <is>
           <t>7834046</t>
         </is>
       </c>
-      <c r="H71" s="7" t="inlineStr">
+      <c r="H71" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -32185,43 +32185,43 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B80" s="7" t="inlineStr">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C80" s="7" t="inlineStr">
+      <c r="C80" s="3" t="inlineStr">
         <is>
           <t>Prickly Pear 72h Hydration &amp; Shine Shampoo
 Champô Figo da Índia Hidratante Cabelo Baço</t>
         </is>
       </c>
-      <c r="D80" s="7" t="inlineStr">
+      <c r="D80" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/prickly-pear-72h-hydration-and-shine-shampoo-355576.html</t>
         </is>
       </c>
-      <c r="E80" s="7" t="inlineStr">
+      <c r="E80" s="3" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="F80" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G80" s="7" t="inlineStr">
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
         <is>
           <t>8067425</t>
         </is>
       </c>
-      <c r="H80" s="7" t="inlineStr">
+      <c r="H80" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -32640,40 +32640,40 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B91" s="7" t="inlineStr">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C91" s="7" t="inlineStr">
+      <c r="C91" s="3" t="inlineStr">
         <is>
           <t>Tamanu &amp; Monoi Nutri-Repair Sun Conditioner
 Condicionador Protetor Solar para Cabelo
 200 ml</t>
         </is>
       </c>
-      <c r="D91" s="7" t="inlineStr">
+      <c r="D91" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/tamanu-and-monoi-nutri-repair-sun-conditioner-7396247.html</t>
         </is>
       </c>
-      <c r="E91" s="7" t="inlineStr"/>
-      <c r="F91" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G91" s="7" t="inlineStr">
+      <c r="E91" s="3" t="inlineStr"/>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
         <is>
           <t>7396247</t>
         </is>
       </c>
-      <c r="H91" s="7" t="inlineStr">
+      <c r="H91" s="3" t="inlineStr">
         <is>
           <t>37%</t>
         </is>
@@ -33761,40 +33761,40 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Head Spa Complexe 5 Essential Oils
 Pré-Champô Estimulante Revitalizante
 50 ml</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/head-spa-complexe-5-essential-oils-5558743.html</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr"/>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>5558743</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -33841,39 +33841,39 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Laca Sytle
 100 ml</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/laca-sytle-7447298.html</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr"/>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr"/>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>7447298</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>29%</t>
         </is>
@@ -34209,40 +34209,40 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Okara Blond Brightening Conditioner Blond Hair
 Condicionador Brilho Louro Natural ou Pintado
 150 ml</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/okara-blond-brightening-conditioner-blond-hair-6760082.html</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr"/>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>6760082</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -34329,40 +34329,40 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>Okara Silver Toning Shampoo
 Champô Violeta Cabelo Branco Grisalho ou Louro
 200 ml</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/okara-silver-toning-shampoo-6759950.html</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr"/>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>6759950</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -34569,40 +34569,40 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>Style Holding Gel Sculpt &amp; Hold
 Gel Cabelo Fixação Sem Resíduos Efeito Wet Look
 150 ml</t>
         </is>
       </c>
-      <c r="D43" s="7" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/style-holding-gel-sculpt-and-hold-7447300.html</t>
         </is>
       </c>
-      <c r="E43" s="7" t="inlineStr"/>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
+      <c r="E43" s="5" t="inlineStr"/>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
         <is>
           <t>7447300</t>
         </is>
       </c>
-      <c r="H43" s="7" t="inlineStr">
+      <c r="H43" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -34649,40 +34649,40 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>Style Modeling Paste
 Pasta para Cabelo Modeladora Fixação Natural
 75 ml</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/style-modeling-paste-7447301.html</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr"/>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="E45" s="5" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>7447301</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
+      <c r="H45" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -34929,40 +34929,40 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C52" s="7" t="inlineStr">
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>Sublime Karité Moisturizing Smooting Mask
 Máscara Hidratante Cabelo Desidratado
 200 ml</t>
         </is>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/sublime-karite-moisturizing-smooting-mask-8109685.html</t>
         </is>
       </c>
-      <c r="E52" s="7" t="inlineStr"/>
-      <c r="F52" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="E52" s="3" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>8109685</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H52" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -35815,40 +35815,40 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B74" s="7" t="inlineStr">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C74" s="7" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>Volumea Volumizing Shampoo
 Champô Volumizador Cabelo Fino sem Volume
 200 ml</t>
         </is>
       </c>
-      <c r="D74" s="7" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/volumea-volumizing-shampoo-5520117.html</t>
         </is>
       </c>
-      <c r="E74" s="7" t="inlineStr"/>
-      <c r="F74" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G74" s="7" t="inlineStr">
+      <c r="E74" s="5" t="inlineStr"/>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
         <is>
           <t>5520117</t>
         </is>
       </c>
-      <c r="H74" s="7" t="inlineStr">
+      <c r="H74" s="5" t="inlineStr">
         <is>
           <t>28%</t>
         </is>
@@ -38042,40 +38042,40 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Protect AC Mattifying Fluid SPF50+
 Protetor Solar Fluido Mate Rosto Pele Oleosa
 40ml</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-ac-mattifying-fluid-spf50-5782463.html</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr"/>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>5782463</t>
         </is>
       </c>
-      <c r="H53" s="7" t="inlineStr">
+      <c r="H53" s="5" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
@@ -38121,40 +38121,40 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Protect Cream SPF50+
 Protetor Solar Creme Rosto Pele Seca
 40 ml</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-cream-spf50-5782489.html</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr"/>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
+      <c r="E55" s="5" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>5782489</t>
         </is>
       </c>
-      <c r="H55" s="7" t="inlineStr">
+      <c r="H55" s="5" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
@@ -38360,40 +38360,40 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C61" s="7" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>Protect Spray SPF50+
 Protetor Solar Spray Rosto Corpo Pele Sensível
 200ml</t>
         </is>
       </c>
-      <c r="D61" s="7" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-spray-spf50-5782493.html</t>
         </is>
       </c>
-      <c r="E61" s="7" t="inlineStr"/>
-      <c r="F61" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G61" s="7" t="inlineStr">
+      <c r="E61" s="5" t="inlineStr"/>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
         <is>
           <t>5782493</t>
         </is>
       </c>
-      <c r="H61" s="7" t="inlineStr">
+      <c r="H61" s="5" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
@@ -39544,11 +39544,7 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>3065975</t>
-        </is>
-      </c>
+      <c r="G26" s="3" t="inlineStr"/>
       <c r="H26" s="3" t="inlineStr">
         <is>
           <t>25%</t>
@@ -41191,7 +41187,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G67" s="5" t="inlineStr"/>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>4219095</t>
+        </is>
+      </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
           <t>25%</t>
@@ -41481,17 +41481,17 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B75" s="7" t="inlineStr">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C75" s="7" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>Eludril
 Ortho Colutório Uso Diário
@@ -41499,23 +41499,23 @@
 500 ml</t>
         </is>
       </c>
-      <c r="D75" s="7" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/ortho-colutorio-uso-diario-7631910.html</t>
         </is>
       </c>
-      <c r="E75" s="7" t="inlineStr"/>
-      <c r="F75" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G75" s="7" t="inlineStr">
+      <c r="E75" s="5" t="inlineStr"/>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
         <is>
           <t>7631910</t>
         </is>
       </c>
-      <c r="H75" s="7" t="inlineStr">
+      <c r="H75" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -41927,17 +41927,17 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="B86" s="7" t="inlineStr">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C86" s="7" t="inlineStr">
+      <c r="C86" s="3" t="inlineStr">
         <is>
           <t>Eludril
 Protect Colutório Uso Diário
@@ -41945,23 +41945,23 @@
 500 ml</t>
         </is>
       </c>
-      <c r="D86" s="7" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-colutorio-uso-diario-7181924.html</t>
         </is>
       </c>
-      <c r="E86" s="7" t="inlineStr"/>
-      <c r="F86" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G86" s="7" t="inlineStr">
+      <c r="E86" s="3" t="inlineStr"/>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
         <is>
           <t>7181924</t>
         </is>
       </c>
-      <c r="H86" s="7" t="inlineStr">
+      <c r="H86" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>

</xml_diff>